<commit_message>
Added functionality to run the CLIGrid web service using lat and long to define a new climate station
</commit_message>
<xml_diff>
--- a/RHEM_template.xlsx
+++ b/RHEM_template.xlsx
@@ -1,30 +1,30 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11114"/>
-  <workbookPr defaultThemeVersion="166925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/GoogleDrive/My Drive/Projects/RHEM/RHEM_batch_app/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gerardo/Library/CloudStorage/GoogleDrive-gerardo@arstucson.net/My Drive/Projects/RHEM/RHEM_batch_app/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{536F90E8-620D-8E43-95DB-5672CC479ECF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60A0F62C-77BF-0346-9CA5-529B2D33C083}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="102400" windowHeight="28300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="34240" yWindow="500" windowWidth="32860" windowHeight="28300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Inputs" sheetId="1" r:id="rId1"/>
     <sheet name="Lookup Tables" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="Uniform">Inputs!$I$33</definedName>
+    <definedName name="Uniform">Inputs!$I$22</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="101">
   <si>
     <t>Scenario Name</t>
   </si>
@@ -258,6 +258,18 @@
   </si>
   <si>
     <t>Concave</t>
+  </si>
+  <si>
+    <t>Scenario Name 2</t>
+  </si>
+  <si>
+    <t>Scenario Description 2</t>
+  </si>
+  <si>
+    <t>CLIGRID</t>
+  </si>
+  <si>
+    <t>32.35, -110.67</t>
   </si>
   <si>
     <t>Units</t>
@@ -466,7 +478,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -492,6 +503,7 @@
     <xf numFmtId="0" fontId="1" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -806,92 +818,92 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BT39"/>
+  <dimension ref="A1:BT28"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="18.1640625" style="8" customWidth="1"/>
-    <col min="2" max="2" width="22" style="8" customWidth="1"/>
-    <col min="3" max="3" width="8.6640625" style="8" customWidth="1"/>
-    <col min="4" max="4" width="10.83203125" style="8" customWidth="1"/>
-    <col min="5" max="5" width="12.6640625" style="9" customWidth="1"/>
-    <col min="6" max="6" width="14.83203125" style="8" customWidth="1"/>
-    <col min="7" max="7" width="7.83203125" style="8" customWidth="1"/>
-    <col min="8" max="8" width="13.33203125" style="8" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="20.5" style="8" customWidth="1"/>
-    <col min="10" max="10" width="11.5" style="8" customWidth="1"/>
-    <col min="11" max="11" width="11.83203125" style="8" customWidth="1"/>
-    <col min="12" max="12" width="15.83203125" style="8" customWidth="1"/>
-    <col min="13" max="13" width="8" style="8" customWidth="1"/>
-    <col min="14" max="14" width="7.83203125" style="8" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="7.33203125" style="8" customWidth="1"/>
-    <col min="16" max="16" width="7.1640625" style="8" customWidth="1"/>
-    <col min="17" max="17" width="8" style="8" customWidth="1"/>
-    <col min="18" max="18" width="11.33203125" style="8" customWidth="1"/>
-    <col min="19" max="19" width="63" style="8" customWidth="1"/>
-    <col min="20" max="20" width="21" style="8" customWidth="1"/>
-    <col min="21" max="21" width="16.83203125" style="8" customWidth="1"/>
-    <col min="22" max="22" width="18.33203125" style="8" customWidth="1"/>
-    <col min="23" max="23" width="16.6640625" style="8" customWidth="1"/>
-    <col min="24" max="24" width="16" style="8" customWidth="1"/>
-    <col min="25" max="25" width="12.33203125" style="8" customWidth="1"/>
+    <col min="1" max="1" width="18.1640625" customWidth="1"/>
+    <col min="2" max="2" width="22" customWidth="1"/>
+    <col min="3" max="3" width="8.6640625" customWidth="1"/>
+    <col min="4" max="4" width="10.83203125" customWidth="1"/>
+    <col min="5" max="5" width="16.6640625" style="8" customWidth="1"/>
+    <col min="6" max="6" width="14.83203125" customWidth="1"/>
+    <col min="7" max="7" width="7.83203125" customWidth="1"/>
+    <col min="8" max="8" width="13.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="20.5" customWidth="1"/>
+    <col min="10" max="10" width="11.5" customWidth="1"/>
+    <col min="11" max="11" width="11.83203125" customWidth="1"/>
+    <col min="12" max="12" width="15.83203125" customWidth="1"/>
+    <col min="13" max="13" width="8" customWidth="1"/>
+    <col min="14" max="14" width="7.83203125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="7.33203125" customWidth="1"/>
+    <col min="16" max="16" width="7.1640625" customWidth="1"/>
+    <col min="17" max="17" width="8" customWidth="1"/>
+    <col min="18" max="18" width="11.33203125" customWidth="1"/>
+    <col min="19" max="19" width="63" customWidth="1"/>
+    <col min="20" max="20" width="21" customWidth="1"/>
+    <col min="21" max="21" width="16.83203125" customWidth="1"/>
+    <col min="22" max="22" width="18.33203125" customWidth="1"/>
+    <col min="23" max="23" width="16.6640625" customWidth="1"/>
+    <col min="24" max="24" width="16" customWidth="1"/>
+    <col min="25" max="25" width="12.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:72" ht="179" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14" t="s">
+      <c r="B1" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="15" t="s">
+      <c r="C1" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="14" t="s">
+      <c r="D1" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="16" t="s">
+      <c r="E1" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="15" t="s">
+      <c r="F1" s="14" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="15" t="s">
+      <c r="G1" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="15" t="s">
+      <c r="H1" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="15" t="s">
+      <c r="I1" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="15" t="s">
+      <c r="J1" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="15" t="s">
+      <c r="K1" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="15" t="s">
+      <c r="L1" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="15" t="s">
+      <c r="M1" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="15" t="s">
+      <c r="N1" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="15" t="s">
+      <c r="O1" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="15" t="s">
+      <c r="P1" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="15" t="s">
+      <c r="Q1" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="15" t="s">
+      <c r="R1" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="13" t="s">
+      <c r="S1" s="12" t="s">
         <v>18</v>
       </c>
       <c r="T1" s="1" t="s">
@@ -927,58 +939,58 @@
       <c r="AD1" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="AE1" s="17" t="s">
+      <c r="AE1" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="AF1" s="17" t="s">
+      <c r="AF1" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="AG1" s="17" t="s">
+      <c r="AG1" s="16" t="s">
         <v>32</v>
       </c>
-      <c r="AH1" s="17" t="s">
+      <c r="AH1" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="AI1" s="17" t="s">
+      <c r="AI1" s="16" t="s">
         <v>34</v>
       </c>
-      <c r="AJ1" s="17" t="s">
+      <c r="AJ1" s="16" t="s">
         <v>35</v>
       </c>
-      <c r="AK1" s="18" t="s">
+      <c r="AK1" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="AL1" s="18" t="s">
+      <c r="AL1" s="17" t="s">
         <v>37</v>
       </c>
-      <c r="AM1" s="18" t="s">
+      <c r="AM1" s="17" t="s">
         <v>38</v>
       </c>
-      <c r="AN1" s="18" t="s">
+      <c r="AN1" s="17" t="s">
         <v>39</v>
       </c>
-      <c r="AO1" s="18" t="s">
+      <c r="AO1" s="17" t="s">
         <v>40</v>
       </c>
-      <c r="AP1" s="18" t="s">
+      <c r="AP1" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="AQ1" s="19" t="s">
+      <c r="AQ1" s="18" t="s">
         <v>42</v>
       </c>
-      <c r="AR1" s="19" t="s">
+      <c r="AR1" s="18" t="s">
         <v>43</v>
       </c>
-      <c r="AS1" s="19" t="s">
+      <c r="AS1" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="AT1" s="19" t="s">
+      <c r="AT1" s="18" t="s">
         <v>45</v>
       </c>
-      <c r="AU1" s="19" t="s">
+      <c r="AU1" s="18" t="s">
         <v>46</v>
       </c>
-      <c r="AV1" s="19" t="s">
+      <c r="AV1" s="18" t="s">
         <v>47</v>
       </c>
       <c r="AW1" s="2" t="s">
@@ -999,66 +1011,66 @@
       <c r="BB1" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="BC1" s="17" t="s">
+      <c r="BC1" s="16" t="s">
         <v>54</v>
       </c>
-      <c r="BD1" s="17" t="s">
+      <c r="BD1" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="BE1" s="17" t="s">
+      <c r="BE1" s="16" t="s">
         <v>56</v>
       </c>
-      <c r="BF1" s="17" t="s">
+      <c r="BF1" s="16" t="s">
         <v>57</v>
       </c>
-      <c r="BG1" s="17" t="s">
+      <c r="BG1" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="BH1" s="17" t="s">
+      <c r="BH1" s="16" t="s">
         <v>59</v>
       </c>
-      <c r="BI1" s="18" t="s">
+      <c r="BI1" s="17" t="s">
         <v>60</v>
       </c>
-      <c r="BJ1" s="18" t="s">
+      <c r="BJ1" s="17" t="s">
         <v>61</v>
       </c>
-      <c r="BK1" s="18" t="s">
+      <c r="BK1" s="17" t="s">
         <v>62</v>
       </c>
-      <c r="BL1" s="18" t="s">
+      <c r="BL1" s="17" t="s">
         <v>63</v>
       </c>
-      <c r="BM1" s="18" t="s">
+      <c r="BM1" s="17" t="s">
         <v>64</v>
       </c>
-      <c r="BN1" s="18" t="s">
+      <c r="BN1" s="17" t="s">
         <v>65</v>
       </c>
-      <c r="BO1" s="19" t="s">
+      <c r="BO1" s="18" t="s">
         <v>66</v>
       </c>
-      <c r="BP1" s="19" t="s">
+      <c r="BP1" s="18" t="s">
         <v>67</v>
       </c>
-      <c r="BQ1" s="19" t="s">
+      <c r="BQ1" s="18" t="s">
         <v>68</v>
       </c>
-      <c r="BR1" s="19" t="s">
+      <c r="BR1" s="18" t="s">
         <v>69</v>
       </c>
-      <c r="BS1" s="19" t="s">
+      <c r="BS1" s="18" t="s">
         <v>70</v>
       </c>
-      <c r="BT1" s="19" t="s">
+      <c r="BT1" s="18" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="2" spans="1:72" x14ac:dyDescent="0.2">
-      <c r="A2" s="10" t="s">
+      <c r="A2" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="B2" s="11" t="s">
+      <c r="B2" s="10" t="s">
         <v>73</v>
       </c>
       <c r="C2">
@@ -1067,430 +1079,279 @@
       <c r="D2" t="s">
         <v>74</v>
       </c>
-      <c r="E2" s="9" t="s">
+      <c r="E2" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="F2" s="12" t="s">
+      <c r="F2" s="11" t="s">
         <v>76</v>
       </c>
-      <c r="G2" s="12">
+      <c r="G2" s="11">
         <v>0</v>
       </c>
       <c r="H2">
         <v>50</v>
       </c>
-      <c r="I2" s="12" t="s">
+      <c r="I2" s="11" t="s">
         <v>77</v>
       </c>
-      <c r="J2" s="11">
-        <v>15</v>
-      </c>
-      <c r="K2" s="11">
+      <c r="J2" s="10">
+        <v>5</v>
+      </c>
+      <c r="K2" s="10">
         <v>0</v>
       </c>
-      <c r="L2" s="11">
+      <c r="L2" s="10">
         <v>0</v>
       </c>
-      <c r="M2" s="11">
+      <c r="M2" s="10">
         <v>20</v>
       </c>
-      <c r="N2" s="11">
+      <c r="N2" s="10">
         <v>0</v>
       </c>
-      <c r="O2" s="11">
+      <c r="O2" s="10">
         <v>0</v>
       </c>
-      <c r="P2" s="11">
+      <c r="P2" s="10">
         <v>0</v>
       </c>
-      <c r="Q2" s="11">
+      <c r="Q2" s="10">
         <v>30</v>
       </c>
-      <c r="R2" s="11">
+      <c r="R2" s="10">
         <v>0</v>
       </c>
-      <c r="T2"/>
-      <c r="U2"/>
-      <c r="V2"/>
-      <c r="W2"/>
-      <c r="X2"/>
-      <c r="Y2"/>
     </row>
     <row r="3" spans="1:72" x14ac:dyDescent="0.2">
-      <c r="A3" s="10"/>
-      <c r="B3" s="11"/>
-      <c r="C3"/>
-      <c r="D3"/>
-      <c r="F3" s="12"/>
-      <c r="G3" s="12"/>
-      <c r="H3"/>
-      <c r="I3" s="12"/>
-      <c r="J3" s="11"/>
-      <c r="K3" s="11"/>
-      <c r="L3" s="11"/>
-      <c r="M3" s="11"/>
-      <c r="N3" s="11"/>
-      <c r="O3" s="11"/>
-      <c r="P3" s="11"/>
-      <c r="Q3" s="11"/>
-      <c r="R3" s="11"/>
-      <c r="T3"/>
-      <c r="U3"/>
-      <c r="V3"/>
-      <c r="W3"/>
-      <c r="X3"/>
-      <c r="Y3"/>
+      <c r="A3" s="19" t="s">
+        <v>78</v>
+      </c>
+      <c r="B3" s="11" t="s">
+        <v>79</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3" t="s">
+        <v>80</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="F3" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="G3" s="11">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>50</v>
+      </c>
+      <c r="I3" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="J3" s="10">
+        <v>5</v>
+      </c>
+      <c r="K3" s="10">
+        <v>0</v>
+      </c>
+      <c r="L3" s="10">
+        <v>0</v>
+      </c>
+      <c r="M3" s="10">
+        <v>20</v>
+      </c>
+      <c r="N3" s="10">
+        <v>0</v>
+      </c>
+      <c r="O3" s="10">
+        <v>0</v>
+      </c>
+      <c r="P3" s="10">
+        <v>0</v>
+      </c>
+      <c r="Q3" s="10">
+        <v>30</v>
+      </c>
+      <c r="R3" s="10">
+        <v>0</v>
+      </c>
     </row>
     <row r="4" spans="1:72" x14ac:dyDescent="0.2">
-      <c r="A4" s="10"/>
-      <c r="B4" s="11"/>
-      <c r="F4" s="12"/>
-      <c r="G4" s="12"/>
-      <c r="I4" s="12"/>
-      <c r="J4" s="11"/>
-      <c r="K4" s="11"/>
-      <c r="L4" s="11"/>
-      <c r="M4" s="11"/>
-      <c r="N4" s="11"/>
-      <c r="O4" s="11"/>
-      <c r="P4" s="11"/>
-      <c r="Q4" s="11"/>
-      <c r="R4" s="11"/>
+      <c r="A4" s="9"/>
+      <c r="B4" s="10"/>
+      <c r="F4" s="11"/>
+      <c r="G4" s="11"/>
+      <c r="I4" s="11"/>
+      <c r="J4" s="10"/>
+      <c r="K4" s="10"/>
+      <c r="L4" s="10"/>
+      <c r="M4" s="10"/>
+      <c r="N4" s="10"/>
+      <c r="O4" s="10"/>
+      <c r="P4" s="10"/>
+      <c r="Q4" s="10"/>
+      <c r="R4" s="10"/>
     </row>
     <row r="5" spans="1:72" x14ac:dyDescent="0.2">
-      <c r="A5" s="10"/>
-      <c r="B5" s="11"/>
-      <c r="F5" s="12"/>
-      <c r="G5" s="12"/>
-      <c r="I5" s="12"/>
-      <c r="J5" s="11"/>
-      <c r="K5" s="11"/>
-      <c r="L5" s="11"/>
-      <c r="M5" s="11"/>
-      <c r="N5" s="11"/>
-      <c r="O5" s="11"/>
-      <c r="P5" s="11"/>
-      <c r="Q5" s="11"/>
-      <c r="R5" s="11"/>
+      <c r="A5" s="9"/>
+      <c r="B5" s="10"/>
+      <c r="F5" s="11"/>
+      <c r="G5" s="11"/>
+      <c r="I5" s="11"/>
+      <c r="J5" s="10"/>
+      <c r="K5" s="10"/>
+      <c r="L5" s="10"/>
+      <c r="M5" s="10"/>
+      <c r="N5" s="10"/>
+      <c r="O5" s="10"/>
+      <c r="P5" s="10"/>
+      <c r="Q5" s="10"/>
+      <c r="R5" s="10"/>
     </row>
     <row r="6" spans="1:72" x14ac:dyDescent="0.2">
-      <c r="A6" s="10"/>
-      <c r="B6" s="11"/>
-      <c r="F6" s="12"/>
-      <c r="G6" s="12"/>
-      <c r="I6" s="12"/>
-      <c r="J6" s="11"/>
-      <c r="K6" s="11"/>
-      <c r="L6" s="11"/>
-      <c r="M6" s="11"/>
-      <c r="N6" s="11"/>
-      <c r="O6" s="11"/>
-      <c r="P6" s="11"/>
-      <c r="Q6" s="11"/>
-      <c r="R6" s="11"/>
+      <c r="A6" s="9"/>
+      <c r="B6" s="10"/>
+      <c r="F6" s="11"/>
+      <c r="G6" s="11"/>
+      <c r="I6" s="11"/>
+      <c r="J6" s="10"/>
+      <c r="K6" s="10"/>
+      <c r="L6" s="10"/>
+      <c r="M6" s="10"/>
+      <c r="N6" s="10"/>
+      <c r="O6" s="10"/>
+      <c r="P6" s="10"/>
+      <c r="Q6" s="10"/>
+      <c r="R6" s="10"/>
     </row>
     <row r="7" spans="1:72" x14ac:dyDescent="0.2">
-      <c r="A7" s="10"/>
-      <c r="B7" s="11"/>
-      <c r="F7" s="12"/>
-      <c r="G7" s="12"/>
-      <c r="I7" s="12"/>
-      <c r="J7" s="11"/>
-      <c r="K7" s="11"/>
-      <c r="L7" s="11"/>
-      <c r="M7" s="11"/>
-      <c r="N7" s="11"/>
-      <c r="O7" s="11"/>
-      <c r="P7" s="11"/>
-      <c r="Q7" s="11"/>
-      <c r="R7" s="11"/>
+      <c r="A7" s="9"/>
+      <c r="B7" s="10"/>
+      <c r="F7" s="11"/>
+      <c r="G7" s="11"/>
+      <c r="I7" s="11"/>
+      <c r="J7" s="10"/>
+      <c r="K7" s="10"/>
+      <c r="L7" s="10"/>
+      <c r="M7" s="10"/>
+      <c r="N7" s="10"/>
+      <c r="O7" s="10"/>
+      <c r="P7" s="10"/>
+      <c r="Q7" s="10"/>
+      <c r="R7" s="10"/>
     </row>
     <row r="8" spans="1:72" x14ac:dyDescent="0.2">
-      <c r="A8" s="10"/>
-      <c r="B8" s="11"/>
-      <c r="F8" s="12"/>
-      <c r="G8" s="12"/>
-      <c r="I8" s="12"/>
-      <c r="J8" s="11"/>
-      <c r="K8" s="11"/>
-      <c r="L8" s="11"/>
-      <c r="M8" s="11"/>
-      <c r="N8" s="11"/>
-      <c r="O8" s="11"/>
-      <c r="P8" s="11"/>
-      <c r="Q8" s="11"/>
-      <c r="R8" s="11"/>
+      <c r="A8" s="9"/>
+      <c r="B8" s="10"/>
+      <c r="F8" s="11"/>
+      <c r="G8" s="11"/>
+      <c r="I8" s="11"/>
+      <c r="J8" s="10"/>
+      <c r="K8" s="10"/>
+      <c r="L8" s="10"/>
+      <c r="M8" s="10"/>
+      <c r="N8" s="10"/>
+      <c r="O8" s="10"/>
+      <c r="P8" s="10"/>
+      <c r="Q8" s="10"/>
+      <c r="R8" s="10"/>
     </row>
     <row r="9" spans="1:72" x14ac:dyDescent="0.2">
-      <c r="A9" s="10"/>
-      <c r="B9" s="11"/>
-      <c r="F9" s="12"/>
-      <c r="G9" s="12"/>
-      <c r="I9" s="12"/>
-      <c r="J9" s="11"/>
-      <c r="K9" s="11"/>
-      <c r="L9" s="11"/>
-      <c r="M9" s="11"/>
-      <c r="N9" s="11"/>
-      <c r="O9" s="11"/>
-      <c r="P9" s="11"/>
-      <c r="Q9" s="11"/>
-      <c r="R9" s="11"/>
+      <c r="A9" s="9"/>
+      <c r="B9" s="10"/>
+      <c r="F9" s="11"/>
+      <c r="G9" s="11"/>
+      <c r="I9" s="11"/>
+      <c r="J9" s="10"/>
+      <c r="K9" s="10"/>
+      <c r="L9" s="10"/>
+      <c r="M9" s="10"/>
+      <c r="N9" s="10"/>
+      <c r="O9" s="10"/>
+      <c r="P9" s="10"/>
+      <c r="Q9" s="10"/>
+      <c r="R9" s="10"/>
     </row>
     <row r="10" spans="1:72" x14ac:dyDescent="0.2">
-      <c r="A10" s="10"/>
-      <c r="B10" s="11"/>
-      <c r="F10" s="12"/>
-      <c r="G10" s="12"/>
-      <c r="I10" s="12"/>
-      <c r="J10" s="11"/>
-      <c r="K10" s="11"/>
-      <c r="L10" s="11"/>
-      <c r="M10" s="11"/>
-      <c r="N10" s="11"/>
-      <c r="O10" s="11"/>
-      <c r="P10" s="11"/>
-      <c r="Q10" s="11"/>
-      <c r="R10" s="11"/>
-    </row>
-    <row r="11" spans="1:72" x14ac:dyDescent="0.2">
-      <c r="A11" s="10"/>
-      <c r="B11" s="11"/>
-      <c r="F11" s="12"/>
-      <c r="G11" s="12"/>
-      <c r="I11" s="12"/>
-      <c r="J11" s="11"/>
-      <c r="K11" s="11"/>
-      <c r="L11" s="11"/>
-      <c r="M11" s="11"/>
-      <c r="N11" s="11"/>
-      <c r="O11" s="11"/>
-      <c r="P11" s="11"/>
-      <c r="Q11" s="11"/>
-      <c r="R11" s="11"/>
-    </row>
-    <row r="12" spans="1:72" x14ac:dyDescent="0.2">
-      <c r="A12" s="10"/>
-      <c r="B12" s="11"/>
-      <c r="F12" s="12"/>
-      <c r="G12" s="12"/>
-      <c r="I12" s="12"/>
-      <c r="J12" s="11"/>
-      <c r="K12" s="11"/>
-      <c r="L12" s="11"/>
-      <c r="M12" s="11"/>
-      <c r="N12" s="11"/>
-      <c r="O12" s="11"/>
-      <c r="P12" s="11"/>
-      <c r="Q12" s="11"/>
-      <c r="R12" s="11"/>
-    </row>
-    <row r="13" spans="1:72" x14ac:dyDescent="0.2">
-      <c r="A13" s="10"/>
-      <c r="B13" s="11"/>
-      <c r="F13" s="12"/>
-      <c r="G13" s="12"/>
-      <c r="I13" s="12"/>
-      <c r="J13" s="11"/>
-      <c r="K13" s="11"/>
-      <c r="L13" s="11"/>
-      <c r="M13" s="11"/>
-      <c r="N13" s="11"/>
-      <c r="O13" s="11"/>
-      <c r="P13" s="11"/>
-      <c r="Q13" s="11"/>
-      <c r="R13" s="11"/>
-    </row>
-    <row r="14" spans="1:72" x14ac:dyDescent="0.2">
-      <c r="A14" s="10"/>
-      <c r="B14" s="11"/>
-      <c r="F14" s="12"/>
-      <c r="G14" s="12"/>
-      <c r="I14" s="12"/>
-      <c r="J14" s="11"/>
-      <c r="K14" s="11"/>
-      <c r="L14" s="11"/>
-      <c r="M14" s="11"/>
-      <c r="N14" s="11"/>
-      <c r="O14" s="11"/>
-      <c r="P14" s="11"/>
-      <c r="Q14" s="11"/>
-      <c r="R14" s="11"/>
-    </row>
-    <row r="15" spans="1:72" x14ac:dyDescent="0.2">
-      <c r="A15" s="10"/>
-      <c r="B15" s="11"/>
-      <c r="F15" s="12"/>
-      <c r="G15" s="12"/>
-      <c r="I15" s="12"/>
-      <c r="J15" s="11"/>
-      <c r="K15" s="11"/>
-      <c r="L15" s="11"/>
-      <c r="M15" s="11"/>
-      <c r="N15" s="11"/>
-      <c r="O15" s="11"/>
-      <c r="P15" s="11"/>
-      <c r="Q15" s="11"/>
-      <c r="R15" s="11"/>
-    </row>
-    <row r="16" spans="1:72" x14ac:dyDescent="0.2">
-      <c r="A16" s="10"/>
-      <c r="B16" s="11"/>
-      <c r="F16" s="12"/>
-      <c r="G16" s="12"/>
-      <c r="I16" s="12"/>
-      <c r="J16" s="11"/>
-      <c r="K16" s="11"/>
-      <c r="L16" s="11"/>
-      <c r="M16" s="11"/>
-      <c r="N16" s="11"/>
-      <c r="O16" s="11"/>
-      <c r="P16" s="11"/>
-      <c r="Q16" s="11"/>
-      <c r="R16" s="11"/>
-    </row>
-    <row r="17" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A17" s="10"/>
-      <c r="B17" s="11"/>
-      <c r="F17" s="12"/>
-      <c r="G17" s="12"/>
-      <c r="I17" s="12"/>
-      <c r="J17" s="11"/>
-      <c r="K17" s="11"/>
-      <c r="L17" s="11"/>
-      <c r="M17" s="11"/>
-      <c r="N17" s="11"/>
-      <c r="O17" s="11"/>
-      <c r="P17" s="11"/>
-      <c r="Q17" s="11"/>
-      <c r="R17" s="11"/>
-    </row>
-    <row r="18" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A18" s="10"/>
-      <c r="B18" s="11"/>
-      <c r="F18" s="12"/>
-      <c r="G18" s="12"/>
-      <c r="I18" s="12"/>
-      <c r="J18" s="11"/>
-      <c r="K18" s="11"/>
-      <c r="L18" s="11"/>
-      <c r="M18" s="11"/>
-      <c r="N18" s="11"/>
-      <c r="O18" s="11"/>
-      <c r="P18" s="11"/>
-      <c r="Q18" s="11"/>
-      <c r="R18" s="11"/>
-    </row>
-    <row r="19" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A19" s="10"/>
-      <c r="B19" s="11"/>
-      <c r="F19" s="12"/>
-      <c r="G19" s="12"/>
-      <c r="I19" s="12"/>
-      <c r="J19" s="11"/>
-      <c r="K19" s="11"/>
-      <c r="L19" s="11"/>
-      <c r="M19" s="11"/>
-      <c r="N19" s="11"/>
-      <c r="O19" s="11"/>
-      <c r="P19" s="11"/>
-      <c r="Q19" s="11"/>
-      <c r="R19" s="11"/>
-    </row>
-    <row r="20" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A20" s="10"/>
-      <c r="B20" s="11"/>
-      <c r="F20" s="12"/>
-      <c r="G20" s="12"/>
-      <c r="I20" s="12"/>
-      <c r="J20" s="11"/>
-      <c r="K20" s="11"/>
-      <c r="L20" s="11"/>
-      <c r="M20" s="11"/>
-      <c r="N20" s="11"/>
-      <c r="O20" s="11"/>
-      <c r="P20" s="11"/>
-      <c r="Q20" s="11"/>
-      <c r="R20" s="11"/>
-    </row>
-    <row r="21" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A21" s="10"/>
-      <c r="B21" s="11"/>
-      <c r="F21" s="12"/>
-      <c r="G21" s="12"/>
-      <c r="I21" s="12"/>
-      <c r="J21" s="11"/>
-      <c r="K21" s="11"/>
-      <c r="L21" s="11"/>
-      <c r="M21" s="11"/>
-      <c r="N21" s="11"/>
-      <c r="O21" s="11"/>
-      <c r="P21" s="11"/>
-      <c r="Q21" s="11"/>
-      <c r="R21" s="11"/>
-    </row>
-    <row r="33" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A33" s="10"/>
-      <c r="B33" s="11"/>
-      <c r="F33" s="12"/>
-      <c r="G33" s="12"/>
-      <c r="I33" s="12"/>
-      <c r="J33" s="11"/>
-      <c r="K33" s="11"/>
-      <c r="L33" s="11"/>
-      <c r="M33" s="11"/>
-      <c r="N33" s="11"/>
-      <c r="O33" s="11"/>
-      <c r="P33" s="11"/>
-      <c r="Q33" s="11"/>
-      <c r="R33" s="11"/>
-    </row>
-    <row r="35" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A35" s="10"/>
-      <c r="B35" s="11"/>
-      <c r="F35" s="12"/>
-      <c r="G35" s="12"/>
-      <c r="I35" s="12"/>
-      <c r="J35" s="11"/>
-      <c r="K35" s="11"/>
-      <c r="L35" s="11"/>
-      <c r="M35" s="11"/>
-      <c r="N35" s="11"/>
-      <c r="O35" s="11"/>
-      <c r="P35" s="11"/>
-      <c r="Q35" s="11"/>
-      <c r="R35" s="11"/>
-    </row>
-    <row r="37" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="A37" s="10"/>
-      <c r="B37" s="11"/>
-      <c r="F37" s="12"/>
-      <c r="G37" s="12"/>
-      <c r="I37" s="12"/>
-      <c r="J37" s="11"/>
-      <c r="K37" s="11"/>
-      <c r="L37" s="11"/>
-      <c r="M37" s="11"/>
-      <c r="N37" s="11"/>
-      <c r="O37" s="11"/>
-      <c r="P37" s="11"/>
-      <c r="Q37" s="11"/>
-      <c r="R37" s="11"/>
-    </row>
-    <row r="39" spans="1:18" x14ac:dyDescent="0.2">
-      <c r="B39" s="11"/>
-      <c r="F39" s="12"/>
-      <c r="G39" s="12"/>
-      <c r="I39" s="12"/>
-      <c r="J39" s="11"/>
-      <c r="K39" s="11"/>
-      <c r="L39" s="11"/>
-      <c r="M39" s="11"/>
-      <c r="N39" s="11"/>
-      <c r="O39" s="11"/>
-      <c r="P39" s="11"/>
-      <c r="Q39" s="11"/>
-      <c r="R39" s="11"/>
+      <c r="A10" s="9"/>
+      <c r="B10" s="10"/>
+      <c r="F10" s="11"/>
+      <c r="G10" s="11"/>
+      <c r="I10" s="11"/>
+      <c r="J10" s="10"/>
+      <c r="K10" s="10"/>
+      <c r="L10" s="10"/>
+      <c r="M10" s="10"/>
+      <c r="N10" s="10"/>
+      <c r="O10" s="10"/>
+      <c r="P10" s="10"/>
+      <c r="Q10" s="10"/>
+      <c r="R10" s="10"/>
+    </row>
+    <row r="22" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A22" s="9"/>
+      <c r="B22" s="10"/>
+      <c r="F22" s="11"/>
+      <c r="G22" s="11"/>
+      <c r="I22" s="11"/>
+      <c r="J22" s="10"/>
+      <c r="K22" s="10"/>
+      <c r="L22" s="10"/>
+      <c r="M22" s="10"/>
+      <c r="N22" s="10"/>
+      <c r="O22" s="10"/>
+      <c r="P22" s="10"/>
+      <c r="Q22" s="10"/>
+      <c r="R22" s="10"/>
+    </row>
+    <row r="24" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A24" s="9"/>
+      <c r="B24" s="10"/>
+      <c r="F24" s="11"/>
+      <c r="G24" s="11"/>
+      <c r="I24" s="11"/>
+      <c r="J24" s="10"/>
+      <c r="K24" s="10"/>
+      <c r="L24" s="10"/>
+      <c r="M24" s="10"/>
+      <c r="N24" s="10"/>
+      <c r="O24" s="10"/>
+      <c r="P24" s="10"/>
+      <c r="Q24" s="10"/>
+      <c r="R24" s="10"/>
+    </row>
+    <row r="26" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="A26" s="9"/>
+      <c r="B26" s="10"/>
+      <c r="F26" s="11"/>
+      <c r="G26" s="11"/>
+      <c r="I26" s="11"/>
+      <c r="J26" s="10"/>
+      <c r="K26" s="10"/>
+      <c r="L26" s="10"/>
+      <c r="M26" s="10"/>
+      <c r="N26" s="10"/>
+      <c r="O26" s="10"/>
+      <c r="P26" s="10"/>
+      <c r="Q26" s="10"/>
+      <c r="R26" s="10"/>
+    </row>
+    <row r="28" spans="1:18" x14ac:dyDescent="0.2">
+      <c r="B28" s="10"/>
+      <c r="F28" s="11"/>
+      <c r="G28" s="11"/>
+      <c r="I28" s="11"/>
+      <c r="J28" s="10"/>
+      <c r="K28" s="10"/>
+      <c r="L28" s="10"/>
+      <c r="M28" s="10"/>
+      <c r="N28" s="10"/>
+      <c r="O28" s="10"/>
+      <c r="P28" s="10"/>
+      <c r="Q28" s="10"/>
+      <c r="R28" s="10"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1503,48 +1364,48 @@
   <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="18" style="8" customWidth="1"/>
-    <col min="2" max="2" width="24.1640625" style="8" customWidth="1"/>
-    <col min="3" max="3" width="24.6640625" style="8" customWidth="1"/>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="24.1640625" customWidth="1"/>
+    <col min="3" max="3" width="24.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="33" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="7"/>
       <c r="B4" s="6" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>77</v>
@@ -1553,37 +1414,37 @@
     <row r="5" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="7"/>
       <c r="B5" s="6" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="7"/>
       <c r="B6" s="6" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="C6" s="5"/>
     </row>
     <row r="7" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="7"/>
       <c r="B7" s="6" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="C7" s="5"/>
     </row>
     <row r="8" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="7"/>
       <c r="B8" s="6" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="C8" s="5"/>
     </row>
     <row r="9" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="7"/>
       <c r="B9" s="6" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="C9" s="5"/>
     </row>
@@ -1597,21 +1458,21 @@
     <row r="11" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="7"/>
       <c r="B11" s="6" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="C11" s="5"/>
     </row>
     <row r="12" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="7"/>
       <c r="B12" s="6" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="C12" s="5"/>
     </row>
     <row r="13" spans="1:3" ht="19" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="7"/>
       <c r="B13" s="6" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="C13" s="5"/>
     </row>

</xml_diff>